<commit_message>
Ajout note concertation 7fcecb13c6c20f80597cc95fbd85ae6a0f42e0f3
</commit_message>
<xml_diff>
--- a/ig/specifications_techniques/StructureDefinition-tddui-bundle.xlsx
+++ b/ig/specifications_techniques/StructureDefinition-tddui-bundle.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>1.0.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-03T08:22:32+00:00</t>
+    <t>2023-10-04T13:47:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>